<commit_message>
docs: clarify unavailable customer rating KPI
</commit_message>
<xml_diff>
--- a/reports/01_KPI_Field_Mapping.xlsx
+++ b/reports/01_KPI_Field_Mapping.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI Field Mapping" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions to Confirm" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GitHub Evidence" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="KPI Field Mapping" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Decisions to Confirm" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Read Me" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="GitHub Evidence" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'KPI Field Mapping'!$A$1:$G$7</definedName>
@@ -728,17 +728,17 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Not yet confirmed</t>
+          <t>Unavailable in verified field inventory</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Locate and verify the rating field, its scale, missingness, and whether it is linked to each order or customer. Avoid treating association as causation.</t>
+          <t>No verified customer-rating field or reliable order-level rating linkage was identified in the current field inventory. Reassess only if a suitable field is found and its scale, missingness, and linkage are validated.</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>Do not calculate this KPI until a suitable rating field and reliable order-level linkage are confirmed; record as unavailable if no such field exists.</t>
+          <t>Do not calculate this KPI unless a suitable rating field and reliable order-level linkage are verified. Otherwise report it as unavailable; do not infer ratings or causation.</t>
         </is>
       </c>
     </row>

</xml_diff>